<commit_message>
Update Jupyter notebook execution counts and uncomment job IDs in evaluation script.
</commit_message>
<xml_diff>
--- a/evaluator_service/evaluation/evaluation_results.xlsx
+++ b/evaluator_service/evaluation/evaluation_results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daves\Desktop\EduFlow\evaluation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daves\Desktop\EduFlow\eduflow\evaluator_service\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58105355-BEC0-45C5-A4FD-51B1C9495FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C44E722-0D33-4BD6-B7B4-6AAA74195412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="99">
   <si>
     <t>Job ID</t>
   </si>
@@ -28,24 +28,21 @@
     <t>Architecture</t>
   </si>
   <si>
-    <t>Topic</t>
-  </si>
-  <si>
-    <t>Learning Focus</t>
-  </si>
-  <si>
-    <t>Target Audience</t>
-  </si>
-  <si>
-    <t>Prompt Lines (Baseline Inputs)</t>
-  </si>
-  <si>
     <t>Duration</t>
   </si>
   <si>
     <t>Number of Docs</t>
   </si>
   <si>
+    <t>Completion Time</t>
+  </si>
+  <si>
+    <t>Total Input Tokens</t>
+  </si>
+  <si>
+    <t>Total Output Tokens</t>
+  </si>
+  <si>
     <t>Custom Matrics</t>
   </si>
   <si>
@@ -59,15 +56,6 @@
   </si>
   <si>
     <t>Eduflow</t>
-  </si>
-  <si>
-    <t>OASIS-Based Clinical Assessment in Home Health</t>
-  </si>
-  <si>
-    <t>Patient assessment, OASIS documentation, clinical decision-making</t>
-  </si>
-  <si>
-    <t>Home health registered nurses</t>
   </si>
   <si>
     <t>{
@@ -216,13 +204,16 @@
     <t>{"architecture": "architecture A", "runs": 3, "mean_scores": {"coherence": 5.0, "dependency_flow": 5.0, "content_progression": 5.0, "non_redundancy": 4.0}, "std_scores": {"coherence": 0.0, "dependency_flow": 0.0, "content_progression": 0.0, "non_redundancy": 0.0}, "overall_mean": 4.75, "run_details": [{"run": 1, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The document sequence demonstrates excellent coherence, with each document logically flowing into the next. The transitions between topics are seamless, and the preview and review sections reinforce the logical progression. Dependency flow is also exemplary, as concepts introduced in earlier documents (e.g., OASIS regulatory framework and assessment techniques) are consistently built upon in later documents (e.g., clinical decision-making and quality improvement). Content progression is outstanding, moving from foundational topics like regulatory requirements to advanced topics like quality improvement and interdisciplinary collaboration. However, there is minor redundancy, particularly in the repeated emphasis on the importance of OASIS accuracy and its impact on quality measures, which could have been streamlined. While this repetition reinforces key points, it slightly detracts from the overall efficiency of the sequence, resulting in a score of 4 for non-redundancy."}, {"run": 2, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document logically flowing from the previous one and building upon the established foundation. The dependency flow is flawless, as concepts introduced early, such as the regulatory framework and OASIS structure, are consistently scaffolded and expanded upon in subsequent documents. Content progression is exemplary, moving systematically from foundational topics to advanced applications, culminating in quality improvement strategies. Non-redundancy is strong, with minimal repetition; while some concepts are revisited, they are reframed in the context of new applications or deeper insights, which adds value rather than redundancy. Overall, the sequence is highly structured and effective in delivering a logical, comprehensive learning experience."}, {"run": 3, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The introductory document sets the foundation, and subsequent documents build logically on the concepts introduced, culminating in quality improvement strategies. Dependency flow is flawless, as concepts introduced early, such as OASIS regulatory requirements and assessment domains, are consistently scaffolded and expanded upon in later documents. Content progression is exemplary, moving from foundational topics like the regulatory framework to advanced topics such as risk stratification and quality improvement. Non-redundancy is strong, with minimal repetition; however, some overlap in the explanation of OASIS items and their impact on quality measures is noticeable across documents, slightly reducing the score in this criterion."}]}</t>
   </si>
   <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>{"job_id": "job-1774534470161", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "learning_focus": "Patient assessment, OASIS documentation, clinical decision-making", "topic": "OASIS-Based Clinical Assessment in Home Health", "target_audience": "Home health registered nurses", "duration": 5, "num_docs": 4, "voice": null}</t>
+  </si>
+  <si>
     <t>job-1774534999912</t>
   </si>
   <si>
     <t>Baseline 1</t>
-  </si>
-  <si>
-    <t>Introduction to OASIS and its role in home health clinical assessment for registered nurses, Conducting comprehensive patient assessments aligned with OASIS requirements in home health settings for registered nurses, Translating clinical observations into accurate OASIS documentation and responses for registered nurses, Handling complex patient scenarios and ensuring compliance with OASIS standards for registered nurses</t>
   </si>
   <si>
     <t>{
@@ -354,6 +345,9 @@
   </si>
   <si>
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. The documents in Sequence X build logically from foundational concepts to advanced topics, with each document clearly flowing from the previous one. Dependency flow is strong, as concepts introduced early are consistently built upon in later documents. Content progression is well-structured, moving from basic regulatory frameworks to advanced clinical decision-making and quality improvement strategies. While both sequences avoid significant redundancy, Sequence X provides a more cohesive and integrated learning experience. Sequence Y, while strong in its own right, lacks the same level of seamless flow and progression, with some minor overlaps in content that slightly detract from its overall effectiveness.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 4}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 5, "Y": 4}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. The documents in Sequence Y are structured as a clear series, with each document building logically on the previous one. The progression from foundational concepts to advanced topics is well-organized, and the series consistently ties assessment techniques to practical applications and quality improvement. Sequence X, while informative, lacks the same level of structured progression and occasionally repeats information unnecessarily, which impacts its non-redundancy score.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 2, "Y": 4}}}, {"run": 3, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. The documents in Sequence X build logically from foundational concepts to advanced applications, with each document clearly flowing from the previous one. Dependency flow is strong, as concepts introduced early are consistently built upon in later documents. Content progression is well-structured, moving from introductory material to practical techniques, clinical decision-making, and quality improvement. While both sequences avoid significant redundancy, Sequence Y occasionally reiterates basic concepts without advancing the discussion, slightly lowering its non-redundancy score. Overall, Sequence X provides a more cohesive and logically structured learning experience.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 4}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 5, "Y": 4}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
+  </si>
+  <si>
+    <t>{"job_id": "job-1774534999912", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to OASIS and its role in home health clinical assessment for registered nurses", "Conducting comprehensive patient assessments aligned with OASIS requirements in home health settings for registered nurses", "Translating clinical observations into accurate OASIS documentation and responses for registered nurses", "Handling complex patient scenarios and ensuring compliance with OASIS standards for registered nurses"], "duration": 5}</t>
   </si>
   <si>
     <t>job-1774544649734</t>
@@ -526,16 +520,10 @@
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, content progression, and non-redundancy. The documents in Sequence Y are structured as a cohesive series, with each document building logically on the previous one. The progression from foundational concepts to advanced applications is clear and systematic, ensuring that readers can follow the learning path effectively. Additionally, Sequence Y avoids unnecessary repetition by focusing on distinct aspects of OASIS assessment in each document, while Sequence X exhibits some redundancy and lacks a clear progression in complexity. Sequence X also struggles with dependency flow, as concepts introduced early are not consistently built upon in later documents.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 2, "Y": 5}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, content progression, and non-redundancy. The documents in Sequence Y are structured as a clear educational series, with each document building logically on the previous one. The progression from foundational concepts to advanced applications is well-defined, and the content avoids unnecessary repetition while reinforcing key ideas. Sequence X, while informative, lacks the same level of structured progression and contains some redundancy across documents, particularly in the repeated explanation of OASIS fundamentals and RN responsibilities.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}, {"run": 3, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, content progression, and non-redundancy. The documents in Sequence Y are structured as a clear educational series, with each document building logically on the previous one. The progression from foundational concepts to advanced applications is well-defined, and the content avoids unnecessary repetition while reinforcing key ideas. Sequence X, while informative, lacks the same level of structured progression and contains some redundancy across documents, particularly in reiterating roles and responsibilities without advancing the discussion significantly.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 2, "Y": 5}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774544649734", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to OASIS and its role in home health clinical assessment for registered nurses", "Conducting comprehensive patient assessments aligned with OASIS requirements in home health settings  for registered nurses", "Translating clinical observations into accurate OASIS documentation and responses  for registered nurses", "Handling complex patient scenarios and ensuring compliance with OASIS standards  for registered nurses"], "duration": 5}</t>
+  </si>
+  <si>
     <t>job-1774545286253</t>
-  </si>
-  <si>
-    <t>Medication Management in Home Health Care</t>
-  </si>
-  <si>
-    <t>Safe medication administration, reconciliation, patient education</t>
-  </si>
-  <si>
-    <t>Home health nurses</t>
   </si>
   <si>
     <t>{
@@ -715,10 +703,10 @@
     <t>{"architecture": "architecture A", "runs": 3, "mean_scores": {"coherence": 5.0, "dependency_flow": 5.0, "content_progression": 5.0, "non_redundancy": 4.33}, "std_scores": {"coherence": 0.0, "dependency_flow": 0.0, "content_progression": 0.0, "non_redundancy": 0.47}, "overall_mean": 4.83, "run_details": [{"run": 1, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The transitions are clear, and the preview sections effectively set up the next topic. Dependency flow is also excellent, as concepts introduced early, such as Medicare requirements and medication reconciliation, are consistently built upon in later documents, culminating in advanced strategies like patient education and sustainable systems. Content progression is logical and well-structured, moving from foundational topics (home health challenges and Medicare requirements) to intermediate (medication reconciliation and administration practices) and finally to advanced topics (patient education and sustainability). Non-redundancy is good, with minor repetition of foundational concepts (e.g., Medicare requirements and the importance of medication safety) across documents, but this repetition serves to reinforce critical points rather than detract from the overall sequence. The series is comprehensive and well-organized, with only slight redundancy in certain sections."}, {"run": 2, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 5}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The introduction in Document 1 sets the stage for the series, and subsequent documents build logically on the foundational concepts introduced. Dependency flow is flawless, as concepts such as medication reconciliation, safe administration practices, and patient education are scaffolded effectively, with each document expanding on prior knowledge. Content progression is ideal, moving from foundational topics (e.g., challenges in home health medication management) to advanced strategies (e.g., high-risk medication protocols and sustainable systems). Non-redundancy is excellent, as each document introduces new information without unnecessary repetition, while reinforcing key concepts in a meaningful way. The series is well-structured, comprehensive, and adheres to the scoring anchors for excellence across all criteria."}, {"run": 3, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The transitions are clear, and the preview sections effectively set up the next topic. Dependency flow is also excellent, as concepts introduced early, such as Medicare requirements and medication reconciliation, are consistently built upon in later documents, culminating in advanced strategies like patient education and sustainable systems. Content progression is logical and well-structured, moving from foundational topics (home health challenges and Medicare requirements) to intermediate (medication reconciliation and administration practices) and finally to advanced topics (patient education and sustainable systems). Non-redundancy is good, with minor repetition of foundational concepts (e.g., Medicare requirements and OASIS documentation) across documents, but this repetition serves to reinforce critical points rather than detract from the overall sequence. The series is highly effective in delivering a comprehensive and structured learning experience for its intended audience."}]}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774545286253", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "learning_focus": "Safe medication administration, reconciliation, patient education", "topic": "Medication Management in Home Health Care", "target_audience": "Home health nurses", "duration": 5, "num_docs": 4, "voice": null}</t>
+  </si>
+  <si>
     <t>job-1774545754239</t>
-  </si>
-  <si>
-    <t>Introduction to medication management principles in home health care for nurses, Best practices for medication reconciliation and avoiding drug interactions in patients for nurses, Educating patients and caregivers about safe medication usage and adherence for nurses, Identifying and managing medication-related risks and adverse effects in home settings for nurses</t>
   </si>
   <si>
     <t>{
@@ -877,6 +865,9 @@
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. The documents in Sequence Y are structured as a cohesive series, with each document building logically on the previous one. The introduction of foundational concepts, followed by systematic methodologies, safe practices, and patient education strategies, ensures a clear progression from basic to advanced topics. Additionally, Sequence Y avoids redundancy by introducing new concepts and techniques in each document, whereas Sequence X exhibits some repetition of information across its documents, particularly in the areas of medication reconciliation and patient education.", "criteria_scores": {"coherence": {"X": 4, "Y": 5}, "dependency_flow": {"X": 4, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}, {"run": 2, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear transitions and previews of upcoming topics. Concepts introduced early are consistently expanded upon, and the sequence moves from foundational principles to advanced practices in a structured manner. Sequence Y, while informative, lacks the same level of interconnectedness and progression, with some redundancy in content and less emphasis on building upon previously introduced concepts.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 3}, "non_redundancy": {"X": 4, "Y": 3}}}, {"run": 3, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear transitions and previews of upcoming topics. Concepts introduced early are consistently expanded upon, and the sequence progresses from foundational principles to advanced practices in a structured manner. Sequence Y, while informative, lacks the same level of interconnectedness and logical progression, with some redundancy in content and less emphasis on building upon previously introduced concepts.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 3}, "non_redundancy": {"X": 4, "Y": 3}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774545754239", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to medication management principles in home health care for nurses", "Best practices for medication reconciliation and avoiding drug interactions in patients for nurses", "Educating patients and caregivers about safe medication usage and adherence for nurses", "Identifying and managing medication-related risks and adverse effects in home settings for nurses"], "duration": 5}</t>
+  </si>
+  <si>
     <t>job-1774547498894</t>
   </si>
   <si>
@@ -1002,13 +993,10 @@
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression compared to Sequence X. Sequence Y is structured as a cohesive series with clear introductions, logical transitions, and consistent reinforcement of prior concepts. It builds systematically from foundational principles to advanced topics, ensuring that each document contributes meaningfully to the overall narrative. Sequence X, while detailed, suffers from some redundancy and less effective content progression, as certain concepts are repeated across documents without significant advancement. Additionally, Sequence Y incorporates more explicit teaching strategies and practical applications, enhancing its overall utility.", "criteria_scores": {"coherence": {"X": 4, "Y": 5}, "dependency_flow": {"X": 4, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 4}}}, {"run": 2, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear transitions and previews of upcoming topics. Concepts introduced early are consistently expanded upon, and the sequence progresses from foundational principles to advanced practices in a structured manner. Sequence Y, while informative, lacks the same level of interconnectedness and progression, with some redundancy and less emphasis on building upon previously introduced concepts.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 3}, "non_redundancy": {"X": 4, "Y": 3}}}, {"run": 3, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, content progression, and non-redundancy compared to Sequence X. Sequence Y is structured as a cohesive series with clear introductions, logical transitions, and consistent reinforcement of key concepts. It builds systematically from foundational principles to advanced topics, ensuring that each document builds upon the previous one. Additionally, Sequence Y avoids unnecessary repetition by introducing new information and perspectives in each document, while Sequence X exhibits some redundancy and less structured progression.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774547498894", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to medication management principles in home health care for nurses", "Best practices for medication reconciliation and avoiding drug interactions in patients for nurses", "Educating patients and caregivers about safe medication usage and adherence for nurses", "Identifying and managing medication-related risks and adverse effects in home settings for nurses"], "duration": 5}</t>
+  </si>
+  <si>
     <t>job-1774548177351</t>
-  </si>
-  <si>
-    <t>Chronic Disease Management in Home Health (COPD and Heart Failure)</t>
-  </si>
-  <si>
-    <t>Symptom monitoring, patient education, early intervention</t>
   </si>
   <si>
     <t>{
@@ -1178,10 +1166,10 @@
     <t>{"architecture": "architecture A", "runs": 3, "mean_scores": {"coherence": 5.0, "dependency_flow": 5.0, "content_progression": 5.0, "non_redundancy": 4.0}, "std_scores": {"coherence": 0.0, "dependency_flow": 0.0, "content_progression": 0.0, "non_redundancy": 0.0}, "overall_mean": 4.75, "run_details": [{"run": 1, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document logically flowing from the previous one and building upon the established foundation. Dependency flow is strong, as concepts introduced early, such as Medicare criteria and OASIS requirements, are consistently scaffolded and expanded upon in later documents. Content progression is exemplary, moving systematically from foundational topics to advanced monitoring, patient education, and care coordination strategies. Non-redundancy is good, with minor repetition of key concepts (e.g., Medicare criteria and OASIS documentation) across documents, but this repetition serves to reinforce critical points rather than detract from the overall content. The series is well-structured and effectively addresses the intended educational goals for home health nurses managing COPD and heart failure patients."}, {"run": 2, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document logically flowing from the previous one and building upon the established foundation. Dependency flow is strong, as concepts introduced early, such as Medicare criteria and OASIS requirements, are consistently scaffolded and expanded upon in later documents. Content progression is exemplary, moving systematically from foundational topics to advanced monitoring, patient education, and care coordination strategies. Non-redundancy is good, with minor repetition of key concepts (e.g., Medicare criteria and OASIS documentation) across documents, which is necessary for reinforcement but slightly reduces the score. Overall, the sequence is highly structured and effective in delivering a logical, comprehensive educational series."}, {"run": 3, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document logically flowing from the previous one and building upon the established foundation. Dependency flow is strong, as concepts introduced early, such as Medicare criteria and OASIS requirements, are consistently scaffolded and expanded upon in later documents. Content progression is exemplary, moving systematically from foundational topics to advanced monitoring, patient education, and care coordination strategies. Non-redundancy is good, with minor repetition of key concepts (e.g., Medicare criteria and OASIS documentation) across documents, but this repetition serves to reinforce critical points rather than detract from the overall content. The series effectively balances depth and breadth while maintaining focus on the intended audience and objectives."}]}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774548177351", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "learning_focus": "Symptom monitoring, patient education, early intervention", "topic": "Chronic Disease Management in Home Health (COPD and Heart Failure)", "target_audience": "Home health nurses", "duration": 5, "num_docs": 4, "voice": null}</t>
+  </si>
+  <si>
     <t>job-1774548651030</t>
-  </si>
-  <si>
-    <t>Overview of chronic disease management for COPD and heart failure in home health patients, Monitoring symptoms and identifying early warning signs in COPD and heart failure patients, Patient education strategies for managing COPD and heart failure at home, Intervention strategies to prevent hospitalization in chronic disease patients</t>
   </si>
   <si>
     <t>{
@@ -1326,6 +1314,9 @@
   </si>
   <si>
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It provides a clear, structured framework for chronic disease management, with each document building logically on the previous one. The introduction of foundational concepts, followed by advanced monitoring, patient education, and care coordination, ensures a logical progression from basic to advanced topics. Additionally, Sequence Y avoids redundancy by focusing on distinct aspects of care in each document, whereas Sequence X exhibits some overlap in content, particularly in patient education and symptom monitoring. Sequence Y also integrates interdisciplinary roles and quality improvement strategies more effectively, enhancing its overall utility and coherence.", "criteria_scores": {"coherence": {"X": 4, "Y": 5}, "dependency_flow": {"X": 4, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It begins with a clear introduction to the series, establishes foundational knowledge, and systematically builds on that foundation with advanced topics, patient education, and care coordination. The documents are explicitly interconnected, with each one previewing the next and reviewing the previous, ensuring a logical flow. Sequence X, while detailed and informative, lacks the same level of structured progression and integration between documents. Additionally, Sequence Y avoids redundancy more effectively by focusing on distinct aspects of chronic disease management in each document, whereas Sequence X repeats certain concepts across multiple documents.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 4}}}, {"run": 3, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It begins with a clear introduction to the series, establishes foundational knowledge, and systematically builds on that foundation with advanced topics, patient education, and care coordination. Each document explicitly references the previous one, ensuring a logical flow and reinforcing dependency between concepts. Sequence X, while detailed and informative, lacks the same level of structured progression and occasionally repeats information unnecessarily, which impacts its non-redundancy score. Sequence Y also integrates quality improvement and interdisciplinary coordination more effectively, aligning with the criteria for content progression and dependency flow.", "criteria_scores": {"coherence": {"X": 4, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 4}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
+  </si>
+  <si>
+    <t>{"job_id": "job-1774548651030", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Overview of chronic disease management for COPD and heart failure in home health patients", "Monitoring symptoms and identifying early warning signs in COPD and heart failure patients", "Patient education strategies for managing COPD and heart failure at home", "Intervention strategies to prevent hospitalization in chronic disease patients"], "duration": 5}</t>
   </si>
   <si>
     <t>job-1774549026730</t>
@@ -1488,13 +1479,10 @@
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document in Sequence X builds systematically on the previous one, with clear transitions and logical development of topics from foundational concepts to advanced strategies. The dependency flow is strong, as concepts introduced early are consistently expanded upon in later documents. Content progression is logical, moving from basic Medicare criteria and assessments to advanced monitoring, patient education, and care coordination. Sequence Y, while well-structured, exhibits some redundancy in its content, particularly in repeating similar points about symptom monitoring and patient education across multiple documents. Additionally, Sequence Y's progression is less clear, with some overlap in topics that could have been better integrated. Sequence X also provides more detailed and actionable insights, enhancing its overall quality.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 4}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 5, "Y": 3}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It begins with a clear introduction to the series, establishes foundational knowledge, and systematically builds toward advanced topics, ensuring logical progression. The documents in Sequence Y are tightly integrated, with each one explicitly referencing and building upon the previous content. Sequence X, while detailed and informative, lacks the same level of structured progression and integration between documents. Additionally, Sequence Y avoids redundancy more effectively, with minimal overlap in content across documents, whereas Sequence X repeats certain concepts and details unnecessarily.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 4}}}, {"run": 3, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It begins with a clear introduction to the series, establishes foundational knowledge, and systematically builds toward advanced topics, ensuring logical progression. The documents in Sequence Y are tightly integrated, with each one explicitly referencing and building upon the previous, which enhances dependency flow. Additionally, Sequence Y avoids redundancy by presenting unique, focused content in each document, whereas Sequence X exhibits some repetition of concepts and lacks the same level of structured progression. Sequence X, while detailed, does not achieve the same level of integration and logical flow as Sequence Y.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774549026730", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Overview of chronic disease management for COPD and heart failure in home health patients", "Monitoring symptoms and identifying early warning signs in COPD and heart failure patients", "Patient education strategies for managing COPD and heart failure at home", "Intervention strategies to prevent hospitalization in chronic disease patients"], "duration": 5}</t>
+  </si>
+  <si>
     <t>job-1774574045744</t>
-  </si>
-  <si>
-    <t>Cognitive Assessment and Care for Alzheimer’s Patients</t>
-  </si>
-  <si>
-    <t>Diagnosis, patient behavior, caregiver support</t>
   </si>
   <si>
     <t>{
@@ -1662,10 +1650,10 @@
     <t>{"architecture": "architecture A", "runs": 3, "mean_scores": {"coherence": 5.0, "dependency_flow": 5.0, "content_progression": 5.0, "non_redundancy": 4.0}, "std_scores": {"coherence": 0.0, "dependency_flow": 0.0, "content_progression": 0.0, "non_redundancy": 0.0}, "overall_mean": 4.75, "run_details": [{"run": 1, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document naturally flowing from the previous one. The introductory sections of each document explicitly reference prior content and set up the next topic, ensuring fluid transitions. Dependency flow is also excellent, as concepts introduced early, such as Alzheimer's progression and Medicare requirements, are consistently built upon in later documents, culminating in practical applications and interdisciplinary coordination. Content progression is logical and well-structured, moving from foundational understanding of Alzheimer's disease to advanced topics like caregiver support and interdisciplinary care coordination. Non-redundancy is good, with minor repetition of key concepts (e.g., Medicare requirements and OASIS documentation) across documents, which is necessary for emphasis but slightly repetitive in certain sections. Overall, the sequence is highly effective and well-organized, with only minor redundancy issues."}, {"run": 2, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document naturally flowing from the previous one. The introductory sections of each document explicitly reference the prior session and preview the next, ensuring seamless transitions. Dependency flow is also excellent, as concepts introduced early, such as Alzheimer's progression and Medicare requirements, are consistently built upon in later documents, culminating in practical applications and interdisciplinary coordination. Content progression is logical and well-structured, moving from foundational understanding of Alzheimer's disease to advanced topics like caregiver support and interdisciplinary care coordination. Non-redundancy is good, with minor repetition of key concepts (e.g., Medicare requirements and OASIS documentation) across documents, which is necessary for emphasis but slightly repetitive. Overall, the sequence is highly effective and well-organized, with only minor redundancy issues."}, {"run": 3, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document naturally flowing from the previous one. The introductory sections of each document explicitly reference prior content and set up the next topic, ensuring fluid transitions. Dependency flow is also excellent, as concepts introduced early, such as Alzheimer's progression and Medicare requirements, are consistently built upon in later documents, culminating in practical applications and interdisciplinary coordination. Content progression is logical and well-structured, moving from foundational understanding of Alzheimer's disease to advanced topics like behavioral management and caregiver support. Non-redundancy is good, with minor repetition of key concepts (e.g., Medicare requirements and OASIS documentation) across documents, but this repetition serves to reinforce critical points rather than detract from the overall content. The sequence effectively balances reinforcement with the introduction of new information, maintaining clarity and focus throughout."}]}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774574045744", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "learning_focus": "Diagnosis, patient behavior, caregiver support", "topic": "Cognitive Assessment and Care for Alzheimer\u2019s Patients", "target_audience": "Home health nurses", "duration": 5, "num_docs": 4, "voice": null}</t>
+  </si>
+  <si>
     <t>job-1774574325545</t>
-  </si>
-  <si>
-    <t>Introduction to Alzheimer’s disease and its clinical diagnosis in home health care for Nurses, Assessing cognitive decline and recognizing symptoms in patients with Alzheimer’s  for Nurses, Managing behavioral and psychological symptoms in Alzheimer’s patients  for Nurses, Supporting caregivers and improving quality of life for patients with cognitive impairment  for Nurses</t>
   </si>
   <si>
     <t>{
@@ -1827,6 +1815,9 @@
   </si>
   <si>
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear transitions and previews of upcoming topics. Concepts introduced early are consistently expanded upon, and the sequence progresses from foundational understanding to advanced strategies in a structured manner. Sequence Y, while informative, lacks the same level of interconnectedness and logical progression, with some redundancy in content and less emphasis on building upon previously introduced concepts.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 4, "Y": 3}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It provides a clear introduction to the series, explicitly outlines the progression of topics, and builds logically from foundational concepts to advanced care strategies. Each document in Sequence Y is interconnected, with explicit references to previous sessions and previews of upcoming ones, ensuring a seamless flow of information. Additionally, Sequence Y avoids redundancy by focusing on distinct aspects of Alzheimer's care in each document, whereas Sequence X repeats certain concepts across multiple documents without adding significant new insights.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 4, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}, {"run": 3, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear transitions and previews of upcoming topics. Concepts introduced early are consistently expanded upon, and the sequence moves from foundational understanding to advanced strategies in a structured manner. Sequence Y, while informative, lacks the same level of interconnectedness and progression, with some redundancy in content and less emphasis on building upon previously introduced concepts.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 4, "Y": 3}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
+  </si>
+  <si>
+    <t>{"job_id": "job-1774574325545", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to Alzheimer\u2019s disease and its clinical diagnosis in home health care for Nurses", "Assessing cognitive decline and recognizing symptoms in patients with Alzheimer\u2019s  for Nurses", "Managing behavioral and psychological symptoms in Alzheimer\u2019s patients  for Nurses", "Supporting caregivers and improving quality of life for patients with cognitive impairment  for Nurses"], "duration": 5}</t>
   </si>
   <si>
     <t>job-1774574626655</t>
@@ -1976,16 +1967,10 @@
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It provides a clear structure with each document building logically on the previous one, starting with foundational concepts and advancing to more complex topics. The series explicitly outlines its progression and ties each session to the next, ensuring a seamless flow of information. Additionally, Sequence Y avoids redundancy by focusing on distinct aspects of Alzheimer's care in each document, whereas Sequence X occasionally repeats information across documents without adding significant new insights.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 4, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It provides a clear structure with each document building logically on the previous one, starting with foundational concepts and advancing to complex topics. The series explicitly outlines its progression and ties each session to the next, ensuring a seamless flow of information. Additionally, Sequence Y avoids redundancy by focusing on distinct aspects of Alzheimer's care in each document, whereas Sequence X occasionally repeats information across documents without adding significant new insights.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}, {"run": 3, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It provides a clear structure with each document building logically on the previous one, starting with foundational concepts and advancing to complex topics. The series explicitly outlines its progression and ties each session to the next, ensuring a seamless flow of information. Additionally, Sequence Y avoids redundancy by focusing on distinct aspects of Alzheimer's care in each document, whereas Sequence X occasionally repeats information across documents without adding significant new insights.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774574626655", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to Alzheimer\u2019s disease and its clinical diagnosis in home health care for Nurses", "Assessing cognitive decline and recognizing symptoms in patients with Alzheimer\u2019s  for Nurses", "Managing behavioral and psychological symptoms in Alzheimer\u2019s patients  for Nurses", "Supporting caregivers and improving quality of life for patients with cognitive impairment  for Nurses"], "duration": 5}</t>
+  </si>
+  <si>
     <t>job-1774590551422</t>
-  </si>
-  <si>
-    <t>Emergency Preparedness in Home Health Care</t>
-  </si>
-  <si>
-    <t>Risk planning, patient safety, emergency protocols</t>
-  </si>
-  <si>
-    <t>Home health staff</t>
   </si>
   <si>
     <t>{
@@ -2176,10 +2161,10 @@
     <t>{"architecture": "architecture A", "runs": 3, "mean_scores": {"coherence": 5.0, "dependency_flow": 5.0, "content_progression": 5.0, "non_redundancy": 4.0}, "std_scores": {"coherence": 0.0, "dependency_flow": 0.0, "content_progression": 0.0, "non_redundancy": 0.0}, "overall_mean": 4.75, "run_details": [{"run": 1, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The transitions are clear, and the content builds logically on prior topics. Dependency flow is also excellent, as concepts introduced early, such as patient vulnerabilities and regulatory requirements, are consistently scaffolded and expanded upon in later documents. Content progression is perfect, moving systematically from foundational topics like regulatory requirements to advanced topics like integration and continuous improvement. Non-redundancy is good, with minor repetition of key points (e.g., Medicare Conditions of Participation and patient vulnerabilities) across documents, but this repetition serves to reinforce critical concepts rather than detract from the overall sequence. The series is well-structured and achieves its educational goals effectively."}, {"run": 2, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The transitions are clear, and the preview sections effectively set up the next topic. Dependency flow is also excellent, as concepts introduced early, such as patient vulnerabilities and regulatory requirements, are consistently built upon in later documents, culminating in actionable strategies and integration into care planning. Content progression is logical and moves from foundational topics (regulatory requirements and patient vulnerabilities) to advanced topics (protocol development, communication strategies, and continuous improvement). Non-redundancy is good, with minor repetition of key concepts such as Medicare Conditions of Participation and patient vulnerabilities, which are necessary for emphasis but slightly overused. Overall, the sequence is highly structured and effective in delivering a comprehensive framework for emergency preparedness in home health settings."}, {"run": 3, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 4}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The transitions are clear, and the content builds logically on prior topics, as evidenced by the consistent references to earlier sessions and previews of upcoming ones. Dependency flow is also excellent, as concepts introduced early, such as patient vulnerabilities and regulatory requirements, are systematically expanded upon in later documents, culminating in actionable protocols and integration strategies. Content progression is perfect, moving from foundational topics like regulatory requirements and patient vulnerabilities to advanced topics like interdisciplinary roles and continuous improvement strategies. Non-redundancy is good, with minor repetition of key points (e.g., Medicare Conditions of Participation and patient vulnerabilities) across documents, but this repetition serves to reinforce critical concepts rather than detract from the overall sequence. The series is well-structured and achieves its educational goals effectively."}]}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774590551422", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "learning_focus": "Risk planning, patient safety, emergency protocols", "topic": "Emergency Preparedness in Home Health Care", "target_audience": "Home health staff", "duration": 5, "num_docs": 4, "voice": null}</t>
+  </si>
+  <si>
     <t>job-1774584736262</t>
-  </si>
-  <si>
-    <t>Introduction to emergency preparedness in home health care settings, Identifying risks and developing emergency plans for home health patients, Ensuring patient safety and continuity of care during emergencies, Roles and responsibilities of home health staff during emergency situations,</t>
   </si>
   <si>
     <t>{
@@ -2329,10 +2314,10 @@
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear references to prior content and a structured progression from foundational concepts to advanced applications. Sequence Y, while informative, lacks the same level of interconnectedness and logical progression, with some redundancy in content and less emphasis on building upon previously introduced concepts.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 4, "Y": 3}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression compared to Sequence X. Sequence Y is structured as a cohesive series, with each document building logically on the previous one, explicitly referencing prior content and previewing upcoming topics. This creates a clear and natural flow of information. Dependency flow is stronger in Sequence Y, as concepts introduced early are consistently expanded upon in later documents, ensuring a logical progression of ideas. Content progression in Sequence Y is more deliberate, moving from foundational concepts to advanced applications in a systematic manner. While both sequences avoid significant redundancy, Sequence X occasionally reiterates similar points across documents without adding substantial new insights, slightly lowering its non-redundancy score.", "criteria_scores": {"coherence": {"X": 4, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 4, "Y": 5}}}, {"run": 3, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression compared to Sequence X. Sequence Y is structured as a cohesive series, with each document building logically on the previous one, and it explicitly references prior and upcoming content to maintain continuity. The content progression in Sequence Y is more deliberate, moving from foundational concepts to advanced applications in a clear and systematic manner. While both sequences avoid significant redundancy, Sequence X occasionally reiterates similar points across documents without adding substantial new insights, slightly lowering its non-redundancy score.", "criteria_scores": {"coherence": {"X": 4, "Y": 5}, "dependency_flow": {"X": 4, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 4, "Y": 5}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774584736262", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to emergency preparedness in home health care settings", "Identifying risks and developing emergency plans for home health patients", "Ensuring patient safety and continuity of care during emergencies", "Roles and responsibilities of home health staff during emergency situations"], "duration": 5}</t>
+  </si>
+  <si>
     <t>job-1774584969330</t>
-  </si>
-  <si>
-    <t>Introduction to emergency preparedness in home health care settings, Identifying risks and developing emergency plans for home health patients, Ensuring patient safety and continuity of care during emergencies, Roles and responsibilities of home health staff during emergency situations</t>
   </si>
   <si>
     <t>{
@@ -2519,16 +2504,10 @@
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear references to prior content and a structured progression from foundational concepts to advanced applications. Sequence Y, while informative, lacks the same level of interconnectedness and logical progression, with some redundancy in content and less emphasis on building upon previously introduced concepts. Sequence X also avoids unnecessary repetition more effectively, ensuring a streamlined and focused presentation of information.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 3}, "non_redundancy": {"X": 5, "Y": 4}}}, {"run": 2, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear references to prior content and a structured progression from foundational concepts to advanced applications. Sequence Y, while informative, lacks the same level of interconnectedness and systematic development, with some gaps in dependency flow and less emphasis on building upon earlier concepts. Additionally, Sequence X avoids redundancy more effectively, presenting unique information in each document without unnecessary repetition.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 5, "Y": 4}}}, {"run": 3, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document builds logically on the previous one, with clear transitions and previews of upcoming topics. The sequence moves systematically from foundational concepts to advanced applications, ensuring a logical progression of content. Additionally, Sequence X avoids redundancy by introducing new information and expanding on prior concepts without unnecessary repetition. Sequence Y, while well-structured, exhibits minor redundancy and less seamless transitions between documents, which slightly impacts its coherence and dependency flow.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 4}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 5, "Y": 4}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774584969330", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Introduction to emergency preparedness in home health care settings", "Identifying risks and developing emergency plans for home health patients", "Ensuring patient safety and continuity of care during emergencies", "Roles and responsibilities of home health staff during emergency situations"], "duration": 5}</t>
+  </si>
+  <si>
     <t>job-1774596210500</t>
-  </si>
-  <si>
-    <t>Regulatory Compliance in Home Health (42 CFR Part 484)</t>
-  </si>
-  <si>
-    <t>Legal requirements, care standards, compliance</t>
-  </si>
-  <si>
-    <t>Home health administrators and nurses</t>
   </si>
   <si>
     <t>{
@@ -2678,10 +2657,10 @@
     <t>{"architecture": "architecture A", "runs": 3, "mean_scores": {"coherence": 5.0, "dependency_flow": 5.0, "content_progression": 5.0, "non_redundancy": 5.0}, "std_scores": {"coherence": 0.0, "dependency_flow": 0.0, "content_progression": 0.0, "non_redundancy": 0.0}, "overall_mean": 5.0, "run_details": [{"run": 1, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 5}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document flowing naturally from the previous one. The introduction of foundational concepts in Document 1 is built upon systematically in subsequent documents, showcasing perfect dependency flow. Content progression is logical, moving from foundational topics like regulatory frameworks to advanced topics such as personnel standards and compliance monitoring. There is no unnecessary repetition across the documents, as each adds distinct and valuable information to the series. The series is well-structured and adheres to the criteria definitions without any noticeable issues."}, {"run": 2, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 5}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document logically flowing from the previous one and building upon the established foundation. Dependency flow is flawless, as concepts introduced early, such as the regulatory framework and Conditions of Participation, are consistently scaffolded and expanded upon in subsequent documents. Content progression is ideal, moving systematically from foundational topics (regulatory framework) to intermediate (patient rights and care planning) and advanced topics (clinical documentation, quality assurance, and personnel standards). Non-redundancy is exemplary, with each document introducing new information and avoiding unnecessary repetition, while reinforcing key points in a manner that supports understanding without redundancy. The series is well-structured and adheres to the criteria perfectly."}, {"run": 3, "scores": {"coherence": 5, "dependency_flow": 5, "content_progression": 5, "non_redundancy": 5}, "reasoning": "The sequence of documents demonstrates excellent coherence, with each document naturally flowing from the previous one and building upon the established foundation. Dependency flow is flawless, as concepts introduced early, such as the regulatory framework and Conditions of Participation, are consistently scaffolded and expanded upon in subsequent documents. Content progression is logical and well-structured, moving from foundational topics like compliance basics to advanced topics such as personnel standards and ongoing compliance monitoring. Non-redundancy is exemplary, with each document introducing new, relevant information without unnecessary repetition, ensuring the series remains engaging and informative throughout."}]}</t>
   </si>
   <si>
+    <t>{"job_id": "job-1774596210500", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "learning_focus": "Legal requirements, care standards, compliance", "topic": "Regulatory Compliance in Home Health (42 CFR Part 484)", "target_audience": "Home health administrators and nurses", "duration": 5, "num_docs": 4, "voice": null}</t>
+  </si>
+  <si>
     <t>job-1774595522117</t>
-  </si>
-  <si>
-    <t>Overview of 42 CFR Part 484 regulations in home health care for health administrators and nurses, Key compliance requirements for patient care and service provision, Documentation and reporting standards under federal regulations, Ensuring ongoing compliance and handling audits in home health agencies</t>
   </si>
   <si>
     <t>{
@@ -2812,6 +2791,9 @@
   </si>
   <si>
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression compared to Sequence X. Sequence Y is structured as a cohesive series with clear introductions, reviews of prior content, and previews of upcoming topics, which enhances its coherence. The dependency flow in Sequence Y is stronger, as each document builds logically on the previous one, reinforcing and expanding on earlier concepts. Content progression in Sequence Y is more deliberate, moving from foundational topics to advanced compliance strategies in a logical sequence. While both sequences exhibit some redundancy, Sequence X has more repeated information across documents, which detracts from its overall effectiveness.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 4}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression compared to Sequence X. Sequence Y is structured as a cohesive series with clear introductions, reviews of prior content, and previews of upcoming topics, which enhances its coherence and logical flow. It builds concepts progressively, starting with foundational regulatory frameworks and advancing to specific compliance areas, ensuring a logical content progression. Additionally, Sequence Y avoids redundancy by presenting unique, focused content in each document, whereas Sequence X exhibits some repetition of information across documents, particularly in regulatory details and compliance requirements.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 5}}}, {"run": 3, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document in Sequence X builds logically on the previous one, with clear transitions and a structured progression from foundational to advanced topics. The dependency flow is strong, as concepts introduced early are consistently expanded upon in later documents. Content progression is logical, moving from regulatory basics to specific compliance areas, clinical documentation, and personnel standards. While both sequences avoid significant redundancy, Sequence X provides more detailed and actionable insights without unnecessary repetition. Sequence Y, while comprehensive, lacks the same level of logical flow and depth in building upon earlier concepts, making it slightly less cohesive and progressive overall.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 4}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 5, "Y": 5}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
+  </si>
+  <si>
+    <t>{"job_id": "job-1774595522117", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Overview of 42 CFR Part 484 regulations in home health care", "Key compliance requirements for patient care and service provision", "Documentation and reporting standards under federal regulations", "Ensuring ongoing compliance and handling audits in home health agencies"], "duration": 5}</t>
   </si>
   <si>
     <t>job-1774596683553</t>
@@ -2967,6 +2949,12 @@
   </si>
   <si>
     <t>{"winner": "sequence_a", "win_counts": {"sequence_a": 3, "sequence_b": 0, "tie": 0}, "win_rate": {"sequence_a": 1.0, "sequence_b": 0.0}, "run_details": [{"run": 1, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression compared to Sequence Y. Sequence X builds a clear narrative, with each document logically flowing into the next, and concepts introduced early are consistently expanded upon in later documents. The content progression in Sequence X is more structured, moving from foundational topics to advanced compliance requirements in a logical manner. While both sequences avoid significant redundancy, Sequence Y occasionally reiterates information without adding new insights, slightly lowering its non-redundancy score.", "criteria_scores": {"coherence": {"X": 5, "Y": 4}, "dependency_flow": {"X": 5, "Y": 4}, "content_progression": {"X": 5, "Y": 4}, "non_redundancy": {"X": 5, "Y": 4}}}, {"run": 2, "order_shown": ["sequence_b", "sequence_a"], "winner": "sequence_a", "reasoning": "Sequence Y demonstrates superior coherence, dependency flow, and content progression. It is structured as a series with clear introductions, reviews, and previews, ensuring each document builds logically on the previous one. The content progresses from foundational concepts to advanced compliance strategies, maintaining a logical flow. Sequence X, while detailed, lacks the same level of structured progression and occasionally repeats information unnecessarily, impacting non-redundancy.", "criteria_scores": {"coherence": {"X": 3, "Y": 5}, "dependency_flow": {"X": 3, "Y": 5}, "content_progression": {"X": 3, "Y": 5}, "non_redundancy": {"X": 3, "Y": 4}}}, {"run": 3, "order_shown": ["sequence_a", "sequence_b"], "winner": "sequence_a", "reasoning": "Sequence X demonstrates superior coherence, dependency flow, and content progression. Each document in Sequence X builds logically on the previous one, with clear transitions and a structured progression from foundational to advanced topics. The dependency flow is strong, as concepts introduced early are consistently expanded upon in later documents. Sequence X also avoids redundancy effectively, with minimal repetition of information. In contrast, Sequence Y, while comprehensive, lacks the same level of coherence and logical progression. The documents in Sequence Y feel more segmented, with less emphasis on building upon previously introduced concepts. Additionally, Sequence Y exhibits some redundancy, particularly in its repeated emphasis on general compliance requirements without adding significant new insights.", "criteria_scores": {"coherence": {"X": 5, "Y": 3}, "dependency_flow": {"X": 5, "Y": 3}, "content_progression": {"X": 5, "Y": 3}, "non_redundancy": {"X": 4, "Y": 3}}}], "consensus": "sequence_a wins with 100% win rate"}</t>
+  </si>
+  <si>
+    <t>{"job_id": "job-1774596683553", "callback_url": "http://host.docker.internal:8001/job-done", "index_id": "0001", "prompts": ["Overview of 42 CFR Part 484 regulations in home health care", "Key compliance requirements for patient care and service provision", "Documentation and reporting standards under federal regulations", "Ensuring ongoing compliance and handling audits in home health agencies"], "duration": 5}</t>
+  </si>
+  <si>
+    <t>Input Parameters</t>
   </si>
 </sst>
 </file>
@@ -3002,11 +2990,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3292,12 +3277,12 @@
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" customWidth="1"/>
-    <col min="6" max="6" width="43" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" customWidth="1"/>
-    <col min="8" max="8" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="30.77734375" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" customWidth="1"/>
+    <col min="7" max="7" width="17.109375" customWidth="1"/>
+    <col min="8" max="8" width="19" customWidth="1"/>
     <col min="9" max="9" width="80.21875" customWidth="1"/>
     <col min="10" max="10" width="66.33203125" customWidth="1"/>
     <col min="11" max="11" width="52.33203125" customWidth="1"/>
@@ -3311,517 +3296,661 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>34</v>
+      </c>
+      <c r="G2">
+        <v>39405</v>
+      </c>
+      <c r="H2">
+        <v>9973</v>
+      </c>
+      <c r="I2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="J2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="K2" t="s">
         <v>14</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2">
-        <v>5</v>
-      </c>
-      <c r="H2">
-        <v>4</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>26</v>
+      </c>
+      <c r="G3">
+        <v>29572</v>
+      </c>
+      <c r="H3">
+        <v>5201</v>
+      </c>
+      <c r="I3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s">
+      <c r="J3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="K3" t="s">
         <v>20</v>
-      </c>
-      <c r="G3">
-        <v>5</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
-      </c>
-      <c r="I3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>28</v>
+      </c>
+      <c r="G4">
+        <v>38306</v>
+      </c>
+      <c r="H4">
+        <v>7520</v>
+      </c>
+      <c r="I4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
+      <c r="J4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4">
-        <v>5</v>
-      </c>
-      <c r="H4">
-        <v>4</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>26</v>
-      </c>
-      <c r="J4" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>34</v>
+      </c>
+      <c r="G5">
+        <v>38608</v>
+      </c>
+      <c r="H5">
+        <v>9541</v>
+      </c>
+      <c r="I5" t="s">
         <v>29</v>
       </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="J5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5">
-        <v>5</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" t="s">
-        <v>34</v>
+      <c r="K5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>26</v>
+      </c>
+      <c r="G6">
+        <v>27969</v>
+      </c>
+      <c r="H6">
+        <v>4850</v>
+      </c>
+      <c r="I6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
         <v>35</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6">
-        <v>5</v>
-      </c>
-      <c r="H6">
-        <v>4</v>
-      </c>
-      <c r="I6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7">
+        <v>28</v>
+      </c>
+      <c r="G7">
+        <v>36614</v>
+      </c>
+      <c r="H7">
+        <v>7286</v>
+      </c>
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" t="s">
         <v>40</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7">
-        <v>5</v>
-      </c>
-      <c r="H7">
-        <v>4</v>
-      </c>
-      <c r="I7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J7" t="s">
-        <v>42</v>
-      </c>
-      <c r="K7" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
         <v>45</v>
       </c>
-      <c r="D8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E8" t="s">
-        <v>32</v>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8">
+        <v>34</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>40186</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>9799</v>
       </c>
       <c r="I8" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="J8" t="s">
-        <v>48</v>
+        <v>44</v>
+      </c>
+      <c r="K8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9">
+        <v>26</v>
+      </c>
+      <c r="G9">
+        <v>29479</v>
+      </c>
+      <c r="H9">
+        <v>4735</v>
+      </c>
+      <c r="I9" t="s">
+        <v>47</v>
+      </c>
+      <c r="J9" t="s">
+        <v>48</v>
+      </c>
+      <c r="K9" t="s">
         <v>49</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9">
-        <v>5</v>
-      </c>
-      <c r="H9">
-        <v>4</v>
-      </c>
-      <c r="I9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J9" t="s">
-        <v>52</v>
-      </c>
-      <c r="K9" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>28</v>
+      </c>
+      <c r="G10">
+        <v>38132</v>
+      </c>
+      <c r="H10">
+        <v>7318</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" t="s">
+        <v>53</v>
+      </c>
+      <c r="K10" t="s">
         <v>54</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" t="s">
-        <v>50</v>
-      </c>
-      <c r="G10">
-        <v>5</v>
-      </c>
-      <c r="H10">
-        <v>4</v>
-      </c>
-      <c r="I10" t="s">
-        <v>55</v>
-      </c>
-      <c r="J10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K10" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
         <v>59</v>
       </c>
-      <c r="D11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E11" t="s">
-        <v>32</v>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11">
+        <v>34</v>
       </c>
       <c r="G11">
-        <v>5</v>
+        <v>40286</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>10107</v>
       </c>
       <c r="I11" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="J11" t="s">
-        <v>62</v>
+        <v>58</v>
+      </c>
+      <c r="K11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12">
+        <v>26</v>
+      </c>
+      <c r="G12">
+        <v>29439</v>
+      </c>
+      <c r="H12">
+        <v>4671</v>
+      </c>
+      <c r="I12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J12" t="s">
+        <v>62</v>
+      </c>
+      <c r="K12" t="s">
         <v>63</v>
-      </c>
-      <c r="B12" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" t="s">
-        <v>64</v>
-      </c>
-      <c r="G12">
-        <v>5</v>
-      </c>
-      <c r="H12">
-        <v>4</v>
-      </c>
-      <c r="I12" t="s">
-        <v>65</v>
-      </c>
-      <c r="J12" t="s">
-        <v>66</v>
-      </c>
-      <c r="K12" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13">
+        <v>28</v>
+      </c>
+      <c r="G13">
+        <v>38302</v>
+      </c>
+      <c r="H13">
+        <v>7464</v>
+      </c>
+      <c r="I13" t="s">
+        <v>66</v>
+      </c>
+      <c r="J13" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" t="s">
         <v>68</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13">
-        <v>5</v>
-      </c>
-      <c r="H13">
-        <v>4</v>
-      </c>
-      <c r="I13" t="s">
-        <v>69</v>
-      </c>
-      <c r="J13" t="s">
-        <v>70</v>
-      </c>
-      <c r="K13" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C14" t="s">
         <v>73</v>
       </c>
-      <c r="D14" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" t="s">
-        <v>75</v>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>4</v>
+      </c>
+      <c r="F14">
+        <v>34</v>
       </c>
       <c r="G14">
-        <v>5</v>
+        <v>40962</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>10397</v>
       </c>
       <c r="I14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="J14" t="s">
-        <v>77</v>
+        <v>72</v>
+      </c>
+      <c r="K14" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
         <v>78</v>
       </c>
-      <c r="B15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F15" t="s">
-        <v>79</v>
+      <c r="D15">
+        <v>5</v>
+      </c>
+      <c r="E15">
+        <v>4</v>
+      </c>
+      <c r="F15">
+        <v>26</v>
       </c>
       <c r="G15">
-        <v>5</v>
+        <v>28916</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>4601</v>
       </c>
       <c r="I15" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="J15" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="K15" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" t="s">
         <v>83</v>
       </c>
-      <c r="B16" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" t="s">
-        <v>84</v>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>4</v>
+      </c>
+      <c r="F16">
+        <v>28</v>
       </c>
       <c r="G16">
-        <v>5</v>
+        <v>37221</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>7035</v>
       </c>
       <c r="I16" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="J16" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="K16" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D17" t="s">
-        <v>90</v>
-      </c>
-      <c r="E17" t="s">
-        <v>91</v>
+        <v>87</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>4</v>
+      </c>
+      <c r="F17">
+        <v>34</v>
       </c>
       <c r="G17">
-        <v>5</v>
+        <v>44208</v>
       </c>
       <c r="H17">
-        <v>4</v>
+        <v>10936</v>
       </c>
       <c r="I17" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="J17" t="s">
-        <v>93</v>
+        <v>86</v>
+      </c>
+      <c r="K17" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" t="s">
-        <v>95</v>
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>26</v>
       </c>
       <c r="G18">
-        <v>5</v>
+        <v>32584</v>
       </c>
       <c r="H18">
-        <v>4</v>
+        <v>4473</v>
       </c>
       <c r="I18" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="J18" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="K18" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>4</v>
+      </c>
+      <c r="F19">
+        <v>28</v>
+      </c>
+      <c r="G19">
+        <v>42185</v>
+      </c>
+      <c r="H19">
+        <v>8039</v>
+      </c>
+      <c r="I19" t="s">
+        <v>94</v>
+      </c>
+      <c r="J19" t="s">
         <v>95</v>
       </c>
-      <c r="G19">
-        <v>5</v>
-      </c>
-      <c r="H19">
-        <v>4</v>
-      </c>
-      <c r="I19" t="s">
-        <v>100</v>
-      </c>
-      <c r="J19" t="s">
-        <v>101</v>
-      </c>
       <c r="K19" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update curriculum plan service and modify evaluation results in Jupyter notebook. Adjusted word count ranges for durations and updated execution counts and output values in the analysis notebook.
</commit_message>
<xml_diff>
--- a/evaluator_service/evaluation/evaluation_results.xlsx
+++ b/evaluator_service/evaluation/evaluation_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daves\Desktop\EduFlow\eduflow\evaluator_service\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C44E722-0D33-4BD6-B7B4-6AAA74195412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D208A9A7-5FF0-4A00-ACE3-F04D988A12ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3340,7 +3340,7 @@
         <v>4</v>
       </c>
       <c r="F2">
-        <v>34</v>
+        <v>223</v>
       </c>
       <c r="G2">
         <v>39405</v>
@@ -3375,7 +3375,7 @@
         <v>4</v>
       </c>
       <c r="F3">
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="G3">
         <v>29572</v>
@@ -3410,7 +3410,7 @@
         <v>4</v>
       </c>
       <c r="F4">
-        <v>28</v>
+        <v>152</v>
       </c>
       <c r="G4">
         <v>38306</v>
@@ -3445,7 +3445,7 @@
         <v>4</v>
       </c>
       <c r="F5">
-        <v>34</v>
+        <v>214</v>
       </c>
       <c r="G5">
         <v>38608</v>
@@ -3480,7 +3480,7 @@
         <v>4</v>
       </c>
       <c r="F6">
-        <v>26</v>
+        <v>106</v>
       </c>
       <c r="G6">
         <v>27969</v>
@@ -3515,7 +3515,7 @@
         <v>4</v>
       </c>
       <c r="F7">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="G7">
         <v>36614</v>
@@ -3550,7 +3550,7 @@
         <v>4</v>
       </c>
       <c r="F8">
-        <v>34</v>
+        <v>227</v>
       </c>
       <c r="G8">
         <v>40186</v>
@@ -3585,7 +3585,7 @@
         <v>4</v>
       </c>
       <c r="F9">
-        <v>26</v>
+        <v>110</v>
       </c>
       <c r="G9">
         <v>29479</v>
@@ -3620,7 +3620,7 @@
         <v>4</v>
       </c>
       <c r="F10">
-        <v>28</v>
+        <v>153</v>
       </c>
       <c r="G10">
         <v>38132</v>
@@ -3655,7 +3655,7 @@
         <v>4</v>
       </c>
       <c r="F11">
-        <v>34</v>
+        <v>224</v>
       </c>
       <c r="G11">
         <v>40286</v>
@@ -3690,7 +3690,7 @@
         <v>4</v>
       </c>
       <c r="F12">
-        <v>26</v>
+        <v>112</v>
       </c>
       <c r="G12">
         <v>29439</v>
@@ -3725,7 +3725,7 @@
         <v>4</v>
       </c>
       <c r="F13">
-        <v>28</v>
+        <v>155</v>
       </c>
       <c r="G13">
         <v>38302</v>
@@ -3760,7 +3760,7 @@
         <v>4</v>
       </c>
       <c r="F14">
-        <v>34</v>
+        <v>230</v>
       </c>
       <c r="G14">
         <v>40962</v>
@@ -3795,7 +3795,7 @@
         <v>4</v>
       </c>
       <c r="F15">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="G15">
         <v>28916</v>
@@ -3830,7 +3830,7 @@
         <v>4</v>
       </c>
       <c r="F16">
-        <v>28</v>
+        <v>157</v>
       </c>
       <c r="G16">
         <v>37221</v>
@@ -3865,7 +3865,7 @@
         <v>4</v>
       </c>
       <c r="F17">
-        <v>34</v>
+        <v>232</v>
       </c>
       <c r="G17">
         <v>44208</v>
@@ -3900,7 +3900,7 @@
         <v>4</v>
       </c>
       <c r="F18">
-        <v>26</v>
+        <v>110</v>
       </c>
       <c r="G18">
         <v>32584</v>
@@ -3935,7 +3935,7 @@
         <v>4</v>
       </c>
       <c r="F19">
-        <v>28</v>
+        <v>156</v>
       </c>
       <c r="G19">
         <v>42185</v>

</xml_diff>

<commit_message>
Update .gitignore to exclude temporary Excel files and adjust word count limits in curriculum plan service. Refactor EduflowGenerator component to utilize job status results directly, and modify Jupyter notebook execution counts for consistency.
</commit_message>
<xml_diff>
--- a/evaluator_service/evaluation/evaluation_results.xlsx
+++ b/evaluator_service/evaluation/evaluation_results.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daves\Desktop\EduFlow\eduflow\evaluator_service\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D208A9A7-5FF0-4A00-ACE3-F04D988A12ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDC7825-EAA4-44E2-ABBA-0F9958E706AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1 (2)" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="104">
   <si>
     <t>Job ID</t>
   </si>
@@ -2955,6 +2956,366 @@
   </si>
   <si>
     <t>Input Parameters</t>
+  </si>
+  <si>
+    <t>{
+  "document_count": 4,
+  "metrics": {
+    "scaffolding_connectivity_score": {
+      "overall": 0.4884,
+      "per_doc": [
+        {
+          "doc_id": 2,
+          "assumptions_count": 15,
+          "satisfied_count": 5,
+          "unsatisfied_concepts": [
+            "Medicare home health benefit eligibility",
+            "Homebound status determination",
+            "CMS Home Health Value-Based Purchasing Model",
+            "Care Compare ratings",
+            "Star Ratings",
+            "OASIS assessment time points",
+            "In-person patient encounters",
+            "Interdisciplinary collaboration in OASIS data collection",
+            "Timely OASIS data submission to CMS",
+            "Clinical record audits for data accuracy"
+          ]
+        },
+        {
+          "doc_id": 3,
+          "assumptions_count": 15,
+          "satisfied_count": 8,
+          "unsatisfied_concepts": [
+            "Care Compare ratings",
+            "Star Ratings",
+            "CMS guidance",
+            "Injectable medication coding",
+            "Levels of assistance in OASIS",
+            "Adult learning principles",
+            "Electronic transmission to CMS"
+          ]
+        },
+        {
+          "doc_id": 4,
+          "assumptions_count": 13,
+          "satisfied_count": 8,
+          "unsatisfied_concepts": [
+            "Comorbidities in patient care",
+            "Cognitive impairments assessment",
+            "Interdisciplinary collaboration",
+            "Drug regimen review",
+            "Professional judgment in nursing"
+          ]
+        }
+      ]
+    },
+    "concept_progression_velocity": {
+      "cpv": 0.8861,
+      "total_unique_concepts": 70,
+      "total_concept_mentions": 79,
+      "repeated_concepts": [
+        "Patient-Driven Groupings Model (PDGM)",
+        "Medication management assessment",
+        "Clinical record integration",
+        "Medicare Conditions of Participation",
+        "Follow-up assessment",
+        "Recertification assessment",
+        "Home Health Quality Reporting Program",
+        "Collaborative data collection",
+        "Comprehensive assessment"
+      ],
+      "per_doc_new_concepts": [
+        20,
+        5,
+        13,
+        8
+      ]
+    },
+    "long_range_scaffolding_depth": {
+      "total_depth": 12,
+      "average_depth": 1.0909,
+      "long_range_links": 1,
+      "total_matched_assumptions": 11,
+      "unmatched_assumptions": 11,
+      "per_doc": [
+        {
+          "doc_id": 2,
+          "matched_assumptions": 4,
+          "depth_sum": 4,
+          "links": [
+            {
+              "concept": "OASIS (Outcome and Assessment Information Set)",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Medicare Conditions of Participation",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Patient-Driven Groupings Model",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Home Health Quality Reporting Program",
+              "introduced_in_doc": 1,
+              "depth": 1
+            }
+          ]
+        },
+        {
+          "doc_id": 3,
+          "matched_assumptions": 3,
+          "depth_sum": 4,
+          "links": [
+            {
+              "concept": "Medicare Conditions of Participation",
+              "introduced_in_doc": 1,
+              "depth": 2
+            },
+            {
+              "concept": "Patient-Driven Groupings Model",
+              "introduced_in_doc": 2,
+              "depth": 1
+            },
+            {
+              "concept": "Environmental assessment",
+              "introduced_in_doc": 2,
+              "depth": 1
+            }
+          ]
+        },
+        {
+          "doc_id": 4,
+          "matched_assumptions": 4,
+          "depth_sum": 4,
+          "links": [
+            {
+              "concept": "Home health care documentation",
+              "introduced_in_doc": 3,
+              "depth": 1
+            },
+            {
+              "concept": "Medication management assessment",
+              "introduced_in_doc": 3,
+              "depth": 1
+            },
+            {
+              "concept": "OASIS-E1 Guidance Manual",
+              "introduced_in_doc": 3,
+              "depth": 1
+            },
+            {
+              "concept": "Regulatory compliance in home health",
+              "introduced_in_doc": 3,
+              "depth": 1
+            }
+          ]
+        }
+      ]
+    }
+  }
+}</t>
+  </si>
+  <si>
+    <t>job-1774645506485</t>
+  </si>
+  <si>
+    <t>set 1</t>
+  </si>
+  <si>
+    <t>job-1774646451702</t>
+  </si>
+  <si>
+    <t>{
+  "document_count": 4,
+  "metrics": {
+    "scaffolding_connectivity_score": {
+      "overall": 0.4651,
+      "per_doc": [
+        {
+          "doc_id": 2,
+          "assumptions_count": 15,
+          "satisfied_count": 8,
+          "unsatisfied_concepts": [
+            "OASIS-E1 guidance manual",
+            "Medication reconciliation process",
+            "Cognitive assessment strategies",
+            "Environmental assessment techniques",
+            "Structured patient interview techniques",
+            "Caregiver integration in assessments",
+            "Hospital discharge summary review"
+          ]
+        },
+        {
+          "doc_id": 3,
+          "assumptions_count": 15,
+          "satisfied_count": 6,
+          "unsatisfied_concepts": [
+            "Care Compare",
+            "Section C (cognitive patterns)",
+            "Section I (active diagnoses)",
+            "M1311 (unhealed pressure ulcers)",
+            "M1324 (stage of pressure ulcer)",
+            "GG0130 (self-care)",
+            "GG0170 (mobility)",
+            "M1033 (risk for hospitalization)",
+            "Medical necessity"
+          ]
+        },
+        {
+          "doc_id": 4,
+          "assumptions_count": 13,
+          "satisfied_count": 6,
+          "unsatisfied_concepts": [
+            "Home Health Quality of Patient Care Star Ratings",
+            "CMS Value-Based Purchasing programs",
+            "Improvement in Dyspnea measure",
+            "Home Health Review and Correct Report",
+            "OASIS Quarterly Q&amp;As",
+            "OASIS-E1 Manual",
+            "attestation signatures for OASIS assessments"
+          ]
+        }
+      ]
+    },
+    "concept_progression_velocity": {
+      "cpv": 0.9375,
+      "total_unique_concepts": 75,
+      "total_concept_mentions": 80,
+      "repeated_concepts": [
+        "Systematic clinical reasoning process",
+        "OASIS assessment data",
+        "Interdisciplinary care planning",
+        "OASIS regulatory framework",
+        "OASIS-based quality measures"
+      ],
+      "per_doc_new_concepts": [
+        20,
+        13,
+        5,
+        10
+      ]
+    },
+    "long_range_scaffolding_depth": {
+      "total_depth": 25,
+      "average_depth": 1.4706,
+      "long_range_links": 6,
+      "total_matched_assumptions": 17,
+      "unmatched_assumptions": 12,
+      "per_doc": [
+        {
+          "doc_id": 2,
+          "matched_assumptions": 6,
+          "depth_sum": 6,
+          "links": [
+            {
+              "concept": "OASIS regulatory framework",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Medicare compliance requirements",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Quality measurement in home health",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Reimbursement decisions in home health",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Functional assessment methods",
+              "introduced_in_doc": 1,
+              "depth": 1
+            },
+            {
+              "concept": "Legal documentation standards for OASIS",
+              "introduced_in_doc": 1,
+              "depth": 1
+            }
+          ]
+        },
+        {
+          "doc_id": 3,
+          "matched_assumptions": 5,
+          "depth_sum": 9,
+          "links": [
+            {
+              "concept": "Patient-Driven Groupings Model (PDGM)",
+              "introduced_in_doc": 1,
+              "depth": 2
+            },
+            {
+              "concept": "Section GG (functional items)",
+              "introduced_in_doc": 1,
+              "depth": 2
+            },
+            {
+              "concept": "Section C (cognitive patterns)",
+              "introduced_in_doc": 2,
+              "depth": 1
+            },
+            {
+              "concept": "Medicare compliance",
+              "introduced_in_doc": 1,
+              "depth": 2
+            },
+            {
+              "concept": "Home Health Conditions of Participation",
+              "introduced_in_doc": 1,
+              "depth": 2
+            }
+          ]
+        },
+        {
+          "doc_id": 4,
+          "matched_assumptions": 6,
+          "depth_sum": 10,
+          "links": [
+            {
+              "concept": "OASIS assessment data",
+              "introduced_in_doc": 3,
+              "depth": 1
+            },
+            {
+              "concept": "evidence-based clinical decisions",
+              "introduced_in_doc": 3,
+              "depth": 1
+            },
+            {
+              "concept": "Care Compare quality measures",
+              "introduced_in_doc": 3,
+              "depth": 1
+            },
+            {
+              "concept": "OASIS-based quality measures",
+              "introduced_in_doc": 3,
+              "depth": 1
+            },
+            {
+              "concept": "internet Quality Improvement and Evaluation System (iQIES)",
+              "introduced_in_doc": 1,
+              "depth": 3
+            },
+            {
+              "concept": "functional status changes",
+              "introduced_in_doc": 1,
+              "depth": 3
+            }
+          ]
+        }
+      ]
+    }
+  }
+}</t>
   </si>
 </sst>
 </file>
@@ -2990,8 +3351,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3957,4 +4319,721 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF344062-7266-4648-BEA7-13666A7CBEDE}">
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.77734375" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" customWidth="1"/>
+    <col min="7" max="7" width="17.109375" customWidth="1"/>
+    <col min="8" max="8" width="19" customWidth="1"/>
+    <col min="9" max="9" width="80.21875" customWidth="1"/>
+    <col min="10" max="10" width="66.33203125" customWidth="1"/>
+    <col min="11" max="11" width="52.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>223</v>
+      </c>
+      <c r="G2">
+        <v>39405</v>
+      </c>
+      <c r="H2">
+        <v>9973</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>119</v>
+      </c>
+      <c r="G3">
+        <v>29572</v>
+      </c>
+      <c r="H3">
+        <v>5201</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>152</v>
+      </c>
+      <c r="G4">
+        <v>38306</v>
+      </c>
+      <c r="H4">
+        <v>7520</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>214</v>
+      </c>
+      <c r="G5">
+        <v>38608</v>
+      </c>
+      <c r="H5">
+        <v>9541</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>106</v>
+      </c>
+      <c r="G6">
+        <v>27969</v>
+      </c>
+      <c r="H6">
+        <v>4850</v>
+      </c>
+      <c r="I6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7">
+        <v>151</v>
+      </c>
+      <c r="G7">
+        <v>36614</v>
+      </c>
+      <c r="H7">
+        <v>7286</v>
+      </c>
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8">
+        <v>227</v>
+      </c>
+      <c r="G8">
+        <v>40186</v>
+      </c>
+      <c r="H8">
+        <v>9799</v>
+      </c>
+      <c r="I8" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" t="s">
+        <v>44</v>
+      </c>
+      <c r="K8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9">
+        <v>110</v>
+      </c>
+      <c r="G9">
+        <v>29479</v>
+      </c>
+      <c r="H9">
+        <v>4735</v>
+      </c>
+      <c r="I9" t="s">
+        <v>47</v>
+      </c>
+      <c r="J9" t="s">
+        <v>48</v>
+      </c>
+      <c r="K9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>153</v>
+      </c>
+      <c r="G10">
+        <v>38132</v>
+      </c>
+      <c r="H10">
+        <v>7318</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" t="s">
+        <v>53</v>
+      </c>
+      <c r="K10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11">
+        <v>224</v>
+      </c>
+      <c r="G11">
+        <v>40286</v>
+      </c>
+      <c r="H11">
+        <v>10107</v>
+      </c>
+      <c r="I11" t="s">
+        <v>57</v>
+      </c>
+      <c r="J11" t="s">
+        <v>58</v>
+      </c>
+      <c r="K11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12">
+        <v>112</v>
+      </c>
+      <c r="G12">
+        <v>29439</v>
+      </c>
+      <c r="H12">
+        <v>4671</v>
+      </c>
+      <c r="I12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J12" t="s">
+        <v>62</v>
+      </c>
+      <c r="K12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13">
+        <v>155</v>
+      </c>
+      <c r="G13">
+        <v>38302</v>
+      </c>
+      <c r="H13">
+        <v>7464</v>
+      </c>
+      <c r="I13" t="s">
+        <v>66</v>
+      </c>
+      <c r="J13" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>4</v>
+      </c>
+      <c r="F14">
+        <v>230</v>
+      </c>
+      <c r="G14">
+        <v>40962</v>
+      </c>
+      <c r="H14">
+        <v>10397</v>
+      </c>
+      <c r="I14" t="s">
+        <v>71</v>
+      </c>
+      <c r="J14" t="s">
+        <v>72</v>
+      </c>
+      <c r="K14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15">
+        <v>5</v>
+      </c>
+      <c r="E15">
+        <v>4</v>
+      </c>
+      <c r="F15">
+        <v>117</v>
+      </c>
+      <c r="G15">
+        <v>28916</v>
+      </c>
+      <c r="H15">
+        <v>4601</v>
+      </c>
+      <c r="I15" t="s">
+        <v>75</v>
+      </c>
+      <c r="J15" t="s">
+        <v>76</v>
+      </c>
+      <c r="K15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>4</v>
+      </c>
+      <c r="F16">
+        <v>157</v>
+      </c>
+      <c r="G16">
+        <v>37221</v>
+      </c>
+      <c r="H16">
+        <v>7035</v>
+      </c>
+      <c r="I16" t="s">
+        <v>80</v>
+      </c>
+      <c r="J16" t="s">
+        <v>81</v>
+      </c>
+      <c r="K16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>4</v>
+      </c>
+      <c r="F17">
+        <v>232</v>
+      </c>
+      <c r="G17">
+        <v>44208</v>
+      </c>
+      <c r="H17">
+        <v>10936</v>
+      </c>
+      <c r="I17" t="s">
+        <v>85</v>
+      </c>
+      <c r="J17" t="s">
+        <v>86</v>
+      </c>
+      <c r="K17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>88</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>110</v>
+      </c>
+      <c r="G18">
+        <v>32584</v>
+      </c>
+      <c r="H18">
+        <v>4473</v>
+      </c>
+      <c r="I18" t="s">
+        <v>89</v>
+      </c>
+      <c r="J18" t="s">
+        <v>90</v>
+      </c>
+      <c r="K18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>4</v>
+      </c>
+      <c r="F19">
+        <v>156</v>
+      </c>
+      <c r="G19">
+        <v>42185</v>
+      </c>
+      <c r="H19">
+        <v>8039</v>
+      </c>
+      <c r="I19" t="s">
+        <v>94</v>
+      </c>
+      <c r="J19" t="s">
+        <v>95</v>
+      </c>
+      <c r="K19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>101</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>100</v>
+      </c>
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" t="s">
+        <v>101</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add faithfulness evaluator and analysis
Introduce faithfulness evaluation features: add a new evaluator (evaluator_service/evaluators/faithfulness_evaluator.py) and an API route (evaluator_service/routes/faithfulness.py), plus a notebook for analysis (evaluator_service/evaluation/faithfulness_analysis.ipynb). Update existing evaluation notebooks (automated_llm_evals.ipynb, downlaod_blos.ipynb) to include additional jobs and captured outputs, and refresh evaluation_results.xlsx. Update Dockerfile to COPY app so the faithfulness code and its imports are available in the image. Minor housekeeping: fix evaluator_service/evaluation/downloaded_jobs path in .gitignore and update main.py and requirements.txt to wire up the new evaluator/route.
</commit_message>
<xml_diff>
--- a/evaluator_service/evaluation/evaluation_results.xlsx
+++ b/evaluator_service/evaluation/evaluation_results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daves\Desktop\EduFlow\eduflow\evaluator_service\evaluation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daves\Desktop\EduFlow\eduflow\evaluator_service\eval_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDC7825-EAA4-44E2-ABBA-0F9958E706AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44A4729-D807-4F81-A6B5-D482FFEA870B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3351,9 +3351,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4399,7 +4398,7 @@
       <c r="H2">
         <v>9973</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" t="s">
         <v>12</v>
       </c>
       <c r="J2" t="s">
@@ -4434,7 +4433,7 @@
       <c r="H3">
         <v>5201</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" t="s">
         <v>18</v>
       </c>
       <c r="J3" t="s">
@@ -5014,7 +5013,7 @@
       <c r="C21" t="s">
         <v>101</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I21" t="s">
         <v>103</v>
       </c>
     </row>
@@ -5028,7 +5027,7 @@
       <c r="C22" t="s">
         <v>101</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="I22" t="s">
         <v>99</v>
       </c>
     </row>

</xml_diff>